<commit_message>
All EU blog business
</commit_message>
<xml_diff>
--- a/scripts/EU_Figures/EU_Figures.xlsx
+++ b/scripts/EU_Figures/EU_Figures.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,36 +414,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>QoQ</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>YoY</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Pre_Covid</t>
         </is>
@@ -478,13 +466,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="E2" t="n">
-        <v>1.16</v>
+        <v>1.15</v>
       </c>
       <c r="F2" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3">
@@ -504,13 +492,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.21</v>
+        <v>-0</v>
       </c>
       <c r="E3" t="n">
-        <v>1.28</v>
+        <v>1.11</v>
       </c>
       <c r="F3" t="n">
-        <v>2.01</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="4">
@@ -530,13 +518,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="E4" t="n">
-        <v>0.71</v>
+        <v>0.55</v>
       </c>
       <c r="F4" t="n">
-        <v>1.94</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="5">
@@ -556,13 +544,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-0.34</v>
+        <v>-0.05</v>
       </c>
       <c r="E5" t="n">
-        <v>0.48</v>
+        <v>0.64</v>
       </c>
       <c r="F5" t="n">
-        <v>1.6</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="6">
@@ -582,19 +570,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.02</v>
+        <v>0.09</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.18</v>
+        <v>0.06</v>
       </c>
       <c r="F6" t="n">
-        <v>1.61</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Labour productivity (per worker)</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -604,17 +592,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.41</v>
+        <v>0.57</v>
       </c>
       <c r="E7" t="n">
-        <v>0.87</v>
+        <v>0.63</v>
       </c>
       <c r="F7" t="n">
-        <v>0.99</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="8">
@@ -630,17 +618,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025Q2</t>
+          <t>2025Q1</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-0.01</v>
+        <v>0.26</v>
       </c>
       <c r="E8" t="n">
-        <v>0.82</v>
+        <v>0.79</v>
       </c>
       <c r="F8" t="n">
-        <v>0.98</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="9">
@@ -656,17 +644,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025Q3</t>
+          <t>2025Q2</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.08</v>
+        <v>-0.11</v>
       </c>
       <c r="E9" t="n">
-        <v>0.72</v>
+        <v>0.63</v>
       </c>
       <c r="F9" t="n">
-        <v>1.06</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="10">
@@ -682,17 +670,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="E10" t="n">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="F10" t="n">
-        <v>1.06</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="11">
@@ -708,23 +696,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>-0.29</v>
+        <v>0.08</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.21</v>
+        <v>0.39</v>
       </c>
       <c r="F11" t="n">
-        <v>0.77</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -734,23 +722,23 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025Q1</t>
+          <t>2026Q1</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.18</v>
+        <v>-0.09</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="F12" t="n">
-        <v>5.17</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -760,17 +748,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025Q2</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.18</v>
+        <v>0.52</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.67</v>
       </c>
       <c r="F13" t="n">
-        <v>5.36</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="14">
@@ -786,17 +774,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2025Q3</t>
+          <t>2025Q1</t>
         </is>
       </c>
       <c r="D14" t="n">
         <v>0.18</v>
       </c>
       <c r="E14" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>5.55</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="15">
@@ -812,17 +800,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q2</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>0.18</v>
       </c>
       <c r="E15" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>5.74</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="16">
@@ -838,23 +826,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="E16" t="n">
-        <v>0.54</v>
+        <v>0.72</v>
       </c>
       <c r="F16" t="n">
-        <v>5.74</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Persons employed</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -864,23 +852,23 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2025Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.76</v>
+        <v>0.09</v>
       </c>
       <c r="E17" t="n">
-        <v>1.59</v>
+        <v>0.63</v>
       </c>
       <c r="F17" t="n">
-        <v>6.88</v>
+        <v>5.64</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Persons employed</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -890,17 +878,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2025Q2</t>
+          <t>2026Q1</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.14</v>
+        <v>0.09</v>
       </c>
       <c r="E18" t="n">
-        <v>1.49</v>
+        <v>0.54</v>
       </c>
       <c r="F18" t="n">
-        <v>7.03</v>
+        <v>5.74</v>
       </c>
     </row>
     <row r="19">
@@ -916,17 +904,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025Q3</t>
+          <t>2025Q1</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3</v>
+        <v>0.62</v>
       </c>
       <c r="E19" t="n">
-        <v>1.47</v>
+        <v>1.52</v>
       </c>
       <c r="F19" t="n">
-        <v>7.36</v>
+        <v>7.02</v>
       </c>
     </row>
     <row r="20">
@@ -942,17 +930,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.14</v>
+        <v>-0.03</v>
       </c>
       <c r="E20" t="n">
-        <v>1.34</v>
+        <v>1.26</v>
       </c>
       <c r="F20" t="n">
-        <v>7.5</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="21">
@@ -968,23 +956,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-0.29</v>
+        <v>0.37</v>
       </c>
       <c r="E21" t="n">
-        <v>0.29</v>
+        <v>1.16</v>
       </c>
       <c r="F21" t="n">
-        <v>7.19</v>
+        <v>7.38</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Total hours worked</t>
+          <t>Real gross value added</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -994,23 +982,23 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2025Q1</t>
+          <t>2025Q4</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="E22" t="n">
-        <v>0.55</v>
+        <v>1.14</v>
       </c>
       <c r="F22" t="n">
-        <v>4.36</v>
+        <v>7.58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Total hours worked</t>
+          <t>Real gross value added</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1020,17 +1008,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2025Q2</t>
+          <t>2026Q1</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-0.09</v>
+        <v>-0.05</v>
       </c>
       <c r="E23" t="n">
-        <v>0.36</v>
+        <v>0.47</v>
       </c>
       <c r="F23" t="n">
-        <v>4.26</v>
+        <v>7.52</v>
       </c>
     </row>
     <row r="24">
@@ -1046,17 +1034,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2025Q3</t>
+          <t>2025Q1</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.36</v>
+        <v>-0.18</v>
       </c>
       <c r="E24" t="n">
-        <v>0.73</v>
+        <v>0.46</v>
       </c>
       <c r="F24" t="n">
-        <v>4.64</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="25">
@@ -1072,17 +1060,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2025Q4</t>
+          <t>2025Q2</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.45</v>
+        <v>0.09</v>
       </c>
       <c r="E25" t="n">
-        <v>0.73</v>
+        <v>0.27</v>
       </c>
       <c r="F25" t="n">
-        <v>5.11</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="26">
@@ -1098,17 +1086,95 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2025Q3</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>-0.27</v>
+        <v>0.27</v>
       </c>
       <c r="E26" t="n">
-        <v>0.45</v>
+        <v>0.64</v>
       </c>
       <c r="F26" t="n">
         <v>4.83</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Total hours worked</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Euro Area</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5.12</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total hours worked</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Euro Area</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5.02</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Total hours worked</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Euro Area</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5.12</v>
       </c>
     </row>
   </sheetData>
@@ -1122,36 +1188,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>QoQ</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>YoY</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Pre_Covid</t>
         </is>
@@ -1160,33 +1226,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Labour productivity (per hour worked)</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Euro Area</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.02</v>
+        <v>-0.1</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.18</v>
+        <v>0.29</v>
       </c>
       <c r="F2" t="n">
-        <v>1.61</v>
+        <v>3.68</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Labour productivity (per worker)</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1196,23 +1262,23 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-0.29</v>
+        <v>0.57</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.21</v>
+        <v>0.63</v>
       </c>
       <c r="F3" t="n">
-        <v>0.77</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1222,23 +1288,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="E4" t="n">
-        <v>0.54</v>
+        <v>0.67</v>
       </c>
       <c r="F4" t="n">
-        <v>5.74</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1248,49 +1314,49 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-0.29</v>
+        <v>0.09</v>
       </c>
       <c r="E5" t="n">
-        <v>0.29</v>
+        <v>0.54</v>
       </c>
       <c r="F5" t="n">
-        <v>7.19</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total hours worked</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Euro Area</t>
+          <t>European Union</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-0.27</v>
+        <v>0.54</v>
       </c>
       <c r="E6" t="n">
-        <v>0.45</v>
+        <v>0.77</v>
       </c>
       <c r="F6" t="n">
-        <v>4.83</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Labour productivity (per hour worked)</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1300,23 +1366,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.12</v>
+        <v>0.55</v>
       </c>
       <c r="E7" t="n">
-        <v>0.15</v>
+        <v>0.92</v>
       </c>
       <c r="F7" t="n">
-        <v>2.91</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Labour productivity (per worker)</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1326,69 +1392,69 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-0.15</v>
+        <v>0.09</v>
       </c>
       <c r="E8" t="n">
-        <v>0.13</v>
+        <v>0.55</v>
       </c>
       <c r="F8" t="n">
-        <v>2.09</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>European Union</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="E9" t="n">
-        <v>0.54</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>5.19</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>European Union</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>-0.18</v>
+        <v>0.01</v>
       </c>
       <c r="E10" t="n">
-        <v>0.64</v>
+        <v>0.52</v>
       </c>
       <c r="F10" t="n">
-        <v>7.84</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="11">
@@ -1399,22 +1465,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>European Union</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D11" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="E11" t="n">
         <v>-0.27</v>
       </c>
-      <c r="E11" t="n">
-        <v>0.46</v>
-      </c>
       <c r="F11" t="n">
-        <v>4.28</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="12">
@@ -1425,22 +1491,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1.06</v>
       </c>
       <c r="E12" t="n">
-        <v>1.2</v>
+        <v>1.45</v>
       </c>
       <c r="F12" t="n">
-        <v>0.35</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="13">
@@ -1451,178 +1517,178 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.49</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.01</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0.01</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>-0.39</v>
       </c>
       <c r="F14" t="n">
-        <v>7.54</v>
+        <v>-1.65</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Total hours worked</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.09</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.36</v>
+        <v>-0.05</v>
       </c>
       <c r="F15" t="n">
-        <v>5.92</v>
+        <v>26.69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Labour productivity (per hour worked)</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.58</v>
+        <v>9.84</v>
       </c>
       <c r="E16" t="n">
-        <v>0.37</v>
+        <v>-1.03</v>
       </c>
       <c r="F16" t="n">
-        <v>1.76</v>
+        <v>18.55</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Labour productivity (per worker)</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.3</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.25</v>
+        <v>11.23</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>-0.09</v>
+        <v>-0.17</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.37</v>
+        <v>-0.33</v>
       </c>
       <c r="F18" t="n">
-        <v>1.05</v>
+        <v>-2.26</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.14</v>
+        <v>-0.15</v>
       </c>
       <c r="E19" t="n">
-        <v>0.39</v>
+        <v>-0.44</v>
       </c>
       <c r="F19" t="n">
-        <v>0.98</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="20">
@@ -1633,22 +1699,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>-0.2</v>
+        <v>0.35</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1.43</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.97</v>
+        <v>10.16</v>
       </c>
     </row>
     <row r="21">
@@ -1659,22 +1725,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-5.44</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>-13.11</v>
+        <v>2.3</v>
       </c>
       <c r="F21" t="n">
-        <v>16.22</v>
+        <v>5.07</v>
       </c>
     </row>
     <row r="22">
@@ -1685,594 +1751,204 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-6.35</v>
+        <v>0.54</v>
       </c>
       <c r="E22" t="n">
-        <v>-13.2</v>
+        <v>1.61</v>
       </c>
       <c r="F22" t="n">
-        <v>8.630000000000001</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-0.72</v>
+        <v>-0.43</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>-0.77</v>
       </c>
       <c r="F23" t="n">
-        <v>18.39</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>-4.48</v>
+        <v>0.61</v>
       </c>
       <c r="E24" t="n">
-        <v>-12.55</v>
+        <v>2.72</v>
       </c>
       <c r="F24" t="n">
-        <v>35.46</v>
+        <v>16.96</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Total hours worked</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>-1.65</v>
+        <v>1.12</v>
       </c>
       <c r="E25" t="n">
-        <v>-0.08</v>
+        <v>3.29</v>
       </c>
       <c r="F25" t="n">
-        <v>10.74</v>
+        <v>15.99</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Labour productivity (per hour worked)</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.19</v>
+        <v>1.04</v>
       </c>
       <c r="F26" t="n">
-        <v>-2.17</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Labour productivity (per worker)</t>
+          <t>Labour productivity (per hour worked)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-0.17</v>
+        <v>-0.15</v>
       </c>
       <c r="E27" t="n">
-        <v>-0.3</v>
+        <v>-0.11</v>
       </c>
       <c r="F27" t="n">
-        <v>0.44</v>
+        <v>2.37</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Persons employed</t>
+          <t>Labour productivity (per worker)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D28" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E28" t="n">
         <v>0.45</v>
       </c>
-      <c r="E28" t="n">
-        <v>1.18</v>
-      </c>
       <c r="F28" t="n">
-        <v>7.01</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Real gross value added</t>
+          <t>Total hours worked</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026Q1</t>
+          <t>2026Q2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.25</v>
+        <v>0.84</v>
       </c>
       <c r="E29" t="n">
-        <v>0.7</v>
+        <v>2.84</v>
       </c>
       <c r="F29" t="n">
-        <v>7.47</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Total hours worked</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F30" t="n">
-        <v>9.779999999999999</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Labour productivity (per hour worked)</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="F31" t="n">
-        <v>3.94</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Labour productivity (per worker)</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>-0.07000000000000001</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1.79</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Persons employed</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F33" t="n">
-        <v>8.039999999999999</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Real gross value added</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="E34" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="F34" t="n">
-        <v>11.03</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Total hours worked</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Netherlands</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="E35" t="n">
-        <v>-0.34</v>
-      </c>
-      <c r="F35" t="n">
-        <v>5.77</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Labour productivity (per hour worked)</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="E36" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="F36" t="n">
-        <v>16.34</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Labour productivity (per worker)</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="E37" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="F37" t="n">
-        <v>14.51</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Real gross value added</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="E38" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="F38" t="n">
-        <v>18.71</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Total hours worked</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="F39" t="n">
-        <v>2.51</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Labour productivity (per hour worked)</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="F40" t="n">
-        <v>2.64</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Labour productivity (per worker)</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="E41" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F41" t="n">
-        <v>-0.02</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Persons employed</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="E42" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="F42" t="n">
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Real gross value added</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="E43" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F43" t="n">
-        <v>12.8</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Total hours worked</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>2026Q1</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>-0.34</v>
-      </c>
-      <c r="E44" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="F44" t="n">
-        <v>8.42</v>
+        <v>9.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>